<commit_message>
Ajout des fichiers HOBO
</commit_message>
<xml_diff>
--- a/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
+++ b/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="4"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="Instruments" sheetId="1" state="visible" r:id="rId3"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="299" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="104">
   <si>
     <t xml:space="preserve">numéro_serie</t>
   </si>
@@ -342,13 +342,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
-    <numFmt numFmtId="167" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -391,12 +390,6 @@
       <name val="Aptos"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
   </fonts>
   <fills count="2">
@@ -441,7 +434,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="8">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -458,11 +451,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -474,11 +463,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -675,8 +660,8 @@
   <dimension ref="A1:I39"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="19.52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="17.52"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="17.95"/>
@@ -708,10 +693,10 @@
       <c r="I1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>21150040</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -726,15 +711,15 @@
       <c r="F2" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G2" s="0" t="s">
+      <c r="G2" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>21150037</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -749,13 +734,12 @@
       <c r="F3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G3" s="0"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>21149850</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -770,13 +754,12 @@
       <c r="F4" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G4" s="0"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>21150035</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -791,13 +774,12 @@
       <c r="F5" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G5" s="0"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>21150041</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -812,13 +794,12 @@
       <c r="F6" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G6" s="0"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>21150042</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -833,13 +814,12 @@
       <c r="F7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G7" s="0"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>21150034</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -854,13 +834,12 @@
       <c r="F8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G8" s="0"/>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>21149855</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C9" s="1" t="s">
@@ -875,13 +854,12 @@
       <c r="F9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="0"/>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>21150036</v>
       </c>
-      <c r="B10" s="0" t="s">
+      <c r="B10" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C10" s="1" t="s">
@@ -896,13 +874,12 @@
       <c r="F10" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G10" s="0"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="1" t="n">
         <v>21150044</v>
       </c>
-      <c r="B11" s="0" t="s">
+      <c r="B11" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -917,15 +894,15 @@
       <c r="F11" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G11" s="0" t="s">
+      <c r="G11" s="1" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
+      <c r="A12" s="1" t="n">
         <v>21150038</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C12" s="1" t="s">
@@ -940,13 +917,12 @@
       <c r="F12" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G12" s="0"/>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="n">
+      <c r="A13" s="1" t="n">
         <v>21149862</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C13" s="1" t="s">
@@ -961,13 +937,12 @@
       <c r="F13" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="n">
+      <c r="A14" s="1" t="n">
         <v>21150038</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C14" s="1" t="s">
@@ -982,13 +957,12 @@
       <c r="F14" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="n">
+      <c r="A15" s="1" t="n">
         <v>21149863</v>
       </c>
-      <c r="B15" s="0" t="s">
+      <c r="B15" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C15" s="1" t="s">
@@ -1003,13 +977,12 @@
       <c r="F15" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="0"/>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="n">
+      <c r="A16" s="1" t="n">
         <v>21149860</v>
       </c>
-      <c r="B16" s="0" t="s">
+      <c r="B16" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C16" s="1" t="s">
@@ -1024,13 +997,12 @@
       <c r="F16" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="0"/>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="n">
+      <c r="A17" s="1" t="n">
         <v>21149846</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C17" s="1" t="s">
@@ -1045,13 +1017,12 @@
       <c r="F17" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="n">
+      <c r="A18" s="1" t="n">
         <v>21150039</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C18" s="1" t="s">
@@ -1066,13 +1037,12 @@
       <c r="F18" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G18" s="0"/>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="n">
+      <c r="A19" s="1" t="n">
         <v>21149859</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C19" s="1" t="s">
@@ -1087,13 +1057,12 @@
       <c r="F19" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G19" s="0"/>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="n">
+      <c r="A20" s="1" t="n">
         <v>21149866</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C20" s="1" t="s">
@@ -1108,13 +1077,12 @@
       <c r="F20" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G20" s="0"/>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="n">
+      <c r="A21" s="1" t="n">
         <v>21149848</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C21" s="1" t="s">
@@ -1129,13 +1097,12 @@
       <c r="F21" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G21" s="0"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="n">
+      <c r="A22" s="1" t="n">
         <v>21149947</v>
       </c>
-      <c r="B22" s="0" t="s">
+      <c r="B22" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C22" s="1" t="s">
@@ -1150,15 +1117,15 @@
       <c r="F22" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G22" s="0" t="s">
+      <c r="G22" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="n">
+      <c r="A23" s="1" t="n">
         <v>21149849</v>
       </c>
-      <c r="B23" s="0" t="s">
+      <c r="B23" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -1173,13 +1140,12 @@
       <c r="F23" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G23" s="0"/>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="n">
+      <c r="A24" s="1" t="n">
         <v>21149852</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C24" s="1" t="s">
@@ -1194,13 +1160,12 @@
       <c r="F24" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G24" s="0"/>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="n">
+      <c r="A25" s="1" t="n">
         <v>21149851</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>34</v>
       </c>
       <c r="C25" s="1" t="s">
@@ -1215,13 +1180,12 @@
       <c r="F25" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G25" s="0"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="n">
+      <c r="A26" s="1" t="n">
         <v>21149845</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>35</v>
       </c>
       <c r="C26" s="1" t="s">
@@ -1236,13 +1200,12 @@
       <c r="F26" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G26" s="0"/>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="n">
+      <c r="A27" s="1" t="n">
         <v>21149854</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C27" s="1" t="s">
@@ -1257,13 +1220,12 @@
       <c r="F27" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G27" s="0"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="n">
+      <c r="A28" s="1" t="n">
         <v>21149853</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C28" s="1" t="s">
@@ -1278,15 +1240,15 @@
       <c r="F28" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G28" s="0" t="s">
+      <c r="G28" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="n">
+      <c r="A29" s="1" t="n">
         <v>21149856</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="B29" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C29" s="1" t="s">
@@ -1301,13 +1263,12 @@
       <c r="F29" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G29" s="0"/>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="n">
+      <c r="A30" s="1" t="n">
         <v>21149843</v>
       </c>
-      <c r="B30" s="0" t="s">
+      <c r="B30" s="1" t="s">
         <v>39</v>
       </c>
       <c r="C30" s="1" t="s">
@@ -1322,15 +1283,15 @@
       <c r="F30" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G30" s="0" t="s">
+      <c r="G30" s="1" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="n">
+      <c r="A31" s="1" t="n">
         <v>21149844</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="B31" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C31" s="1" t="s">
@@ -1345,13 +1306,12 @@
       <c r="F31" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G31" s="0"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="n">
+      <c r="A32" s="1" t="n">
         <v>21150045</v>
       </c>
-      <c r="B32" s="0" t="s">
+      <c r="B32" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C32" s="1" t="s">
@@ -1366,13 +1326,12 @@
       <c r="F32" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G32" s="0"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="n">
+      <c r="A33" s="1" t="n">
         <v>21150043</v>
       </c>
-      <c r="B33" s="0" t="s">
+      <c r="B33" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C33" s="1" t="s">
@@ -1387,15 +1346,15 @@
       <c r="F33" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G33" s="0" t="s">
+      <c r="G33" s="1" t="s">
         <v>40</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="n">
+      <c r="A34" s="1" t="n">
         <v>21150046</v>
       </c>
-      <c r="B34" s="0" t="s">
+      <c r="B34" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C34" s="1" t="s">
@@ -1410,15 +1369,15 @@
       <c r="F34" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G34" s="0" t="s">
+      <c r="G34" s="1" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="n">
+      <c r="A35" s="1" t="n">
         <v>21150047</v>
       </c>
-      <c r="B35" s="0" t="s">
+      <c r="B35" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C35" s="1" t="s">
@@ -1433,15 +1392,15 @@
       <c r="F35" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G35" s="0" t="s">
+      <c r="G35" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="n">
+      <c r="A36" s="1" t="n">
         <v>21150048</v>
       </c>
-      <c r="B36" s="0" t="s">
+      <c r="B36" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C36" s="1" t="s">
@@ -1456,15 +1415,15 @@
       <c r="F36" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G36" s="0" t="s">
+      <c r="G36" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="n">
+      <c r="A37" s="1" t="n">
         <v>21149857</v>
       </c>
-      <c r="B37" s="0" t="s">
+      <c r="B37" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C37" s="1" t="s">
@@ -1479,13 +1438,12 @@
       <c r="F37" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G37" s="0"/>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="n">
+      <c r="A38" s="1" t="n">
         <v>21149858</v>
       </c>
-      <c r="B38" s="0" t="s">
+      <c r="B38" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C38" s="1" t="s">
@@ -1500,15 +1458,15 @@
       <c r="F38" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G38" s="0" t="s">
+      <c r="G38" s="1" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="n">
+      <c r="A39" s="1" t="n">
         <v>21150032</v>
       </c>
-      <c r="B39" s="0" t="s">
+      <c r="B39" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C39" s="1" t="s">
@@ -1523,7 +1481,7 @@
       <c r="F39" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="G39" s="0" t="s">
+      <c r="G39" s="1" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1547,8 +1505,8 @@
   <dimension ref="A1:E39"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31.88"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="25.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.88"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="33.67"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="85.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="21.38"/>
@@ -1568,7 +1526,7 @@
       <c r="E1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B2" s="4" t="n">
@@ -1579,7 +1537,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B3" s="4" t="n">
@@ -1590,7 +1548,7 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B4" s="4" t="n">
@@ -1601,7 +1559,7 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B5" s="4" t="n">
@@ -1612,7 +1570,7 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B6" s="4" t="n">
@@ -1623,7 +1581,7 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B7" s="4" t="n">
@@ -1634,7 +1592,7 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B8" s="4" t="n">
@@ -1645,7 +1603,7 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B9" s="4" t="n">
@@ -1656,7 +1614,7 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B10" s="4" t="n">
@@ -1667,7 +1625,7 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B11" s="4" t="n">
@@ -1678,7 +1636,7 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B12" s="4" t="n">
@@ -1689,7 +1647,7 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B13" s="4" t="n">
@@ -1700,7 +1658,7 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B14" s="4" t="n">
@@ -1711,7 +1669,7 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B15" s="4" t="n">
@@ -1722,7 +1680,7 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B16" s="4" t="n">
@@ -1733,7 +1691,7 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B17" s="4" t="n">
@@ -1744,7 +1702,7 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B18" s="4" t="n">
@@ -1755,7 +1713,7 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B19" s="4" t="n">
@@ -1766,7 +1724,7 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B20" s="4" t="n">
@@ -1777,7 +1735,7 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B21" s="4" t="n">
@@ -1788,7 +1746,7 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B22" s="4" t="n">
@@ -1799,7 +1757,7 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B23" s="4" t="n">
@@ -1810,7 +1768,7 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B24" s="4" t="n">
@@ -1821,7 +1779,7 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B25" s="4" t="n">
@@ -1832,7 +1790,7 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B26" s="4" t="n">
@@ -1843,7 +1801,7 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B27" s="4" t="n">
@@ -1854,7 +1812,7 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B28" s="4" t="n">
@@ -1865,7 +1823,7 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="A29" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B29" s="4" t="n">
@@ -1876,7 +1834,7 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B30" s="4" t="n">
@@ -1887,7 +1845,7 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B31" s="4" t="n">
@@ -1898,7 +1856,7 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+      <c r="A32" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B32" s="4" t="n">
@@ -1909,7 +1867,7 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+      <c r="A33" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B33" s="4" t="n">
@@ -1920,7 +1878,7 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+      <c r="A34" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B34" s="4" t="n">
@@ -1931,7 +1889,7 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="A35" s="1" t="s">
         <v>45</v>
       </c>
       <c r="B35" s="4"/>
@@ -1940,7 +1898,7 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
+      <c r="A36" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B36" s="4"/>
@@ -1949,7 +1907,7 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+      <c r="A37" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B37" s="4" t="n">
@@ -1960,7 +1918,7 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
+      <c r="A38" s="1" t="s">
         <v>49</v>
       </c>
       <c r="B38" s="4"/>
@@ -1969,7 +1927,7 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
+      <c r="A39" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B39" s="4" t="n">
@@ -2024,8 +1982,8 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2044,7 +2002,7 @@
     <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.6"/>
@@ -2065,12 +2023,345 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B2" s="7"/>
-      <c r="C2" s="6"/>
+      <c r="A2" s="0" t="n">
+        <v>-0.09653415444</v>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>55</v>
+      </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="7"/>
-      <c r="C3" s="6"/>
+      <c r="A3" s="0" t="n">
+        <v>-0.08044650796</v>
+      </c>
+      <c r="B3" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C3" s="5" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="0" t="n">
+        <v>0.05317033367</v>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="0" t="n">
+        <v>-0.0570970766</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="0" t="n">
+        <v>-0.05486268126</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="0" t="n">
+        <v>-0.03564688129</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="0" t="n">
+        <v>-0.1518354392</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="0" t="n">
+        <v>-0.07340816262</v>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="0" t="n">
+        <v>-0.06167758706</v>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="0" t="n">
+        <v>0.005689432592</v>
+      </c>
+      <c r="B11" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="0" t="n">
+        <v>0.06635326621</v>
+      </c>
+      <c r="B12" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="0" t="n">
+        <v>0.06724702435</v>
+      </c>
+      <c r="B13" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="0" t="n">
+        <v>0.1786316323</v>
+      </c>
+      <c r="B14" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="0" t="n">
+        <v>0.0766314848</v>
+      </c>
+      <c r="B15" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="0" t="n">
+        <v>0.1915911253</v>
+      </c>
+      <c r="B16" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="0" t="n">
+        <v>0.1263467812</v>
+      </c>
+      <c r="B17" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C17" s="5" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="0" t="n">
+        <v>0.1069075417</v>
+      </c>
+      <c r="B18" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C18" s="5" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="0" t="n">
+        <v>0.1437750649</v>
+      </c>
+      <c r="B19" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="0" t="n">
+        <v>-0.02615070108</v>
+      </c>
+      <c r="B20" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="0" t="n">
+        <v>0.1119349312</v>
+      </c>
+      <c r="B21" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="0" t="n">
+        <v>-0.1126218009</v>
+      </c>
+      <c r="B22" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="0" t="n">
+        <v>-0.09698103351</v>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C23" s="5" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="0" t="n">
+        <v>0.006136311661</v>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="0" t="n">
+        <v>-0.02324598713</v>
+      </c>
+      <c r="B25" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="0" t="n">
+        <v>-0.05519784056</v>
+      </c>
+      <c r="B26" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="0" t="n">
+        <v>-0.0697214103</v>
+      </c>
+      <c r="B27" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="0" t="n">
+        <v>-0.138987666</v>
+      </c>
+      <c r="B28" s="6" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B29" s="6"/>
+      <c r="C29" s="5"/>
+    </row>
+    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B30" s="6"/>
+      <c r="C30" s="5"/>
+    </row>
+    <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B31" s="6"/>
+      <c r="C31" s="5"/>
+    </row>
+    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B32" s="6"/>
+      <c r="C32" s="5"/>
+    </row>
+    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="6"/>
+      <c r="C33" s="5"/>
+    </row>
+    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B34" s="6"/>
+      <c r="C34" s="5"/>
+    </row>
+    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B35" s="6"/>
+      <c r="C35" s="5"/>
+    </row>
+    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B36" s="6"/>
+      <c r="C36" s="5"/>
+    </row>
+    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B37" s="6"/>
+      <c r="C37" s="5"/>
+    </row>
+    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B38" s="6"/>
+      <c r="C38" s="5"/>
+    </row>
+    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B39" s="6"/>
+      <c r="C39" s="5"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2111,10 +2402,10 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B2" s="9" t="n">
+      <c r="A2" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B2" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C2" s="1" t="s">
@@ -2125,10 +2416,10 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B3" s="9" t="n">
+      <c r="A3" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B3" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C3" s="1" t="s">
@@ -2139,10 +2430,10 @@
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B4" s="9" t="n">
+      <c r="A4" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B4" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C4" s="1" t="s">
@@ -2153,10 +2444,10 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B5" s="9" t="n">
+      <c r="A5" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B5" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C5" s="1" t="s">
@@ -2167,10 +2458,10 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B6" s="9" t="n">
+      <c r="A6" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B6" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C6" s="1" t="s">
@@ -2181,10 +2472,10 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B7" s="9" t="n">
+      <c r="A7" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B7" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C7" s="1" t="s">
@@ -2195,10 +2486,10 @@
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B8" s="9" t="n">
+      <c r="A8" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B8" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C8" s="1" t="s">
@@ -2209,10 +2500,10 @@
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B9" s="9" t="n">
+      <c r="A9" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B9" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C9" s="1" t="s">
@@ -2223,10 +2514,10 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B10" s="9" t="n">
+      <c r="A10" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B10" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C10" s="1" t="s">
@@ -2237,10 +2528,10 @@
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B11" s="9" t="n">
+      <c r="A11" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B11" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C11" s="1" t="s">
@@ -2251,10 +2542,10 @@
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B12" s="9" t="n">
+      <c r="A12" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B12" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C12" s="1" t="s">
@@ -2265,10 +2556,10 @@
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B13" s="9" t="n">
+      <c r="A13" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B13" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C13" s="1" t="s">
@@ -2279,10 +2570,10 @@
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B14" s="9" t="n">
+      <c r="A14" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B14" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C14" s="1" t="s">
@@ -2293,10 +2584,10 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B15" s="9" t="n">
+      <c r="A15" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B15" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C15" s="1" t="s">
@@ -2307,10 +2598,10 @@
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B16" s="9" t="n">
+      <c r="A16" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B16" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C16" s="1" t="s">
@@ -2321,10 +2612,10 @@
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B17" s="9" t="n">
+      <c r="A17" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B17" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C17" s="1" t="s">
@@ -2335,10 +2626,10 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B18" s="9" t="n">
+      <c r="A18" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B18" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C18" s="1" t="s">
@@ -2349,10 +2640,10 @@
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B19" s="9" t="n">
+      <c r="A19" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B19" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C19" s="1" t="s">
@@ -2363,10 +2654,10 @@
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B20" s="9" t="n">
+      <c r="A20" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B20" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C20" s="1" t="s">
@@ -2377,10 +2668,10 @@
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B21" s="9" t="n">
+      <c r="A21" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B21" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C21" s="1" t="s">
@@ -2391,10 +2682,10 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B22" s="9" t="n">
+      <c r="A22" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B22" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C22" s="1" t="s">
@@ -2405,10 +2696,10 @@
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B23" s="9" t="n">
+      <c r="A23" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B23" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C23" s="1" t="s">
@@ -2419,10 +2710,10 @@
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B24" s="9" t="n">
+      <c r="A24" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B24" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C24" s="1" t="s">
@@ -2433,10 +2724,10 @@
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B25" s="9" t="n">
+      <c r="A25" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B25" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C25" s="1" t="s">
@@ -2447,10 +2738,10 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B26" s="9" t="n">
+      <c r="A26" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B26" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C26" s="1" t="s">
@@ -2461,10 +2752,10 @@
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B27" s="9" t="n">
+      <c r="A27" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B27" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C27" s="1" t="s">
@@ -2475,10 +2766,10 @@
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B28" s="9" t="n">
+      <c r="A28" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B28" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C28" s="1" t="s">
@@ -2489,10 +2780,10 @@
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B29" s="9" t="n">
+      <c r="A29" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B29" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C29" s="1" t="s">
@@ -2503,10 +2794,10 @@
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B30" s="9" t="n">
+      <c r="A30" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B30" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C30" s="1" t="s">
@@ -2517,10 +2808,10 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B31" s="9" t="n">
+      <c r="A31" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B31" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C31" s="1" t="s">
@@ -2531,10 +2822,10 @@
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B32" s="9" t="n">
+      <c r="A32" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B32" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C32" s="1" t="s">
@@ -2545,10 +2836,10 @@
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B33" s="9" t="n">
+      <c r="A33" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B33" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C33" s="1" t="s">
@@ -2559,10 +2850,10 @@
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B34" s="9" t="n">
+      <c r="A34" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B34" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C34" s="1" t="s">
@@ -2573,10 +2864,10 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B35" s="9" t="n">
+      <c r="A35" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B35" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C35" s="1" t="s">
@@ -2587,10 +2878,10 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B36" s="9" t="n">
+      <c r="A36" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B36" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C36" s="1" t="s">
@@ -2601,10 +2892,10 @@
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B37" s="9" t="n">
+      <c r="A37" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B37" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C37" s="1" t="s">
@@ -2615,10 +2906,10 @@
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B38" s="9" t="n">
+      <c r="A38" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B38" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C38" s="1" t="s">
@@ -2629,10 +2920,10 @@
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B39" s="9" t="n">
+      <c r="A39" s="6" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B39" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C39" s="1" t="s">

</xml_diff>

<commit_message>
Ajout des métadonnées des instruments TMS4 et Dendromètre
</commit_message>
<xml_diff>
--- a/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
+++ b/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="117">
   <si>
     <t xml:space="preserve">numéro_serie</t>
   </si>
@@ -179,6 +179,21 @@
     <t xml:space="preserve">HOBO_n°38</t>
   </si>
   <si>
+    <t xml:space="preserve">TMS4_n°0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOMST</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMS4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dendro_n°0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dendro</t>
+  </si>
+  <si>
     <t xml:space="preserve">identifiant_instrument (num_instrument)</t>
   </si>
   <si>
@@ -300,6 +315,30 @@
   </si>
   <si>
     <t xml:space="preserve">capteur de température du HOBO n°38</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01/09/2023</t>
+  </si>
+  <si>
+    <t xml:space="preserve">capteur de température à -6cm du sol du TMS4 n°0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">capteur de température à 2cm du sol du TMS4 n°0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">capteur de température à 15cm du sol du TMS4 n°0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">capteur de conductivité du TMS4 n°0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">01/03/2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">capteur de température du Dendromètre n°0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">capteur de variation de diamètre du Dendromètre n°0</t>
   </si>
   <si>
     <t xml:space="preserve">id_initial</t>
@@ -347,7 +386,7 @@
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -387,6 +426,13 @@
     <font>
       <sz val="12"/>
       <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color rgb="FF000000"/>
       <name val="Aptos"/>
       <family val="0"/>
       <charset val="1"/>
@@ -434,7 +480,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -457,6 +503,10 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -654,11 +704,10 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I39"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:I41"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="19.52"/>
@@ -1483,6 +1532,34 @@
       </c>
       <c r="G39" s="1" t="s">
         <v>31</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="n">
+        <v>95224601</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="n">
+        <v>92261195</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="D41" s="0" t="s">
+        <v>55</v>
       </c>
     </row>
   </sheetData>
@@ -1499,28 +1576,27 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:E45"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.38"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="33.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="43.25"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="85.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="21.38"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="D1" s="2"/>
       <c r="E1" s="3"/>
@@ -1533,7 +1609,7 @@
         <v>45412</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1544,7 +1620,7 @@
         <v>45412</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1555,7 +1631,7 @@
         <v>45412</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1566,7 +1642,7 @@
         <v>45412</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1577,7 +1653,7 @@
         <v>45412</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1588,7 +1664,7 @@
         <v>45412</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1599,7 +1675,7 @@
         <v>45412</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1610,7 +1686,7 @@
         <v>45412</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1621,7 +1697,7 @@
         <v>45412</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1632,7 +1708,7 @@
         <v>45412</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1643,7 +1719,7 @@
         <v>45412</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1654,7 +1730,7 @@
         <v>45412</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1665,7 +1741,7 @@
         <v>45412</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1676,7 +1752,7 @@
         <v>45412</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1687,7 +1763,7 @@
         <v>45412</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1698,7 +1774,7 @@
         <v>45412</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1709,7 +1785,7 @@
         <v>45412</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1720,7 +1796,7 @@
         <v>45451</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1731,7 +1807,7 @@
         <v>45451</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1742,7 +1818,7 @@
         <v>45451</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1753,7 +1829,7 @@
         <v>45451</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1764,7 +1840,7 @@
         <v>45451</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1775,7 +1851,7 @@
         <v>45451</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1786,7 +1862,7 @@
         <v>45451</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1797,7 +1873,7 @@
         <v>45451</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1808,7 +1884,7 @@
         <v>45451</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1819,7 +1895,7 @@
         <v>45451</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1830,7 +1906,7 @@
         <v>45451</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1841,7 +1917,7 @@
         <v>46098</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1852,7 +1928,7 @@
         <v>45451</v>
       </c>
       <c r="C31" s="5" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1863,7 +1939,7 @@
         <v>45451</v>
       </c>
       <c r="C32" s="5" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1874,7 +1950,7 @@
         <v>46098</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1885,7 +1961,7 @@
         <v>45451</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1894,7 +1970,7 @@
       </c>
       <c r="B35" s="4"/>
       <c r="C35" s="5" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1903,7 +1979,7 @@
       </c>
       <c r="B36" s="4"/>
       <c r="C36" s="5" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1914,7 +1990,7 @@
         <v>45451</v>
       </c>
       <c r="C37" s="5" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1923,7 +1999,7 @@
       </c>
       <c r="B38" s="4"/>
       <c r="C38" s="5" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1934,7 +2010,73 @@
         <v>45451</v>
       </c>
       <c r="C39" s="5" t="s">
-        <v>91</v>
+        <v>96</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B40" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C40" s="5" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B41" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C41" s="5" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B42" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B43" s="6" t="s">
+        <v>97</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B44" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B45" s="6" t="s">
+        <v>102</v>
+      </c>
+      <c r="C45" s="5" t="s">
+        <v>104</v>
       </c>
     </row>
   </sheetData>
@@ -1951,11 +2093,10 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E3"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="37"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="35.48"/>
@@ -1966,19 +2107,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>92</v>
+        <v>105</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>93</v>
+        <v>106</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>95</v>
+        <v>108</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>96</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1999,11 +2140,10 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:C39"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14.6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="24.62"/>
@@ -2013,354 +2153,354 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>97</v>
+        <v>110</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>98</v>
+        <v>111</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="1" t="n">
         <v>-0.09653415444</v>
       </c>
-      <c r="B2" s="6" t="n">
+      <c r="B2" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="1" t="n">
         <v>-0.08044650796</v>
       </c>
-      <c r="B3" s="6" t="n">
+      <c r="B3" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
+      <c r="A4" s="1" t="n">
         <v>0.05317033367</v>
       </c>
-      <c r="B4" s="6" t="n">
+      <c r="B4" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
+      <c r="A5" s="1" t="n">
         <v>-0.0570970766</v>
       </c>
-      <c r="B5" s="6" t="n">
+      <c r="B5" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
+      <c r="A6" s="1" t="n">
         <v>-0.05486268126</v>
       </c>
-      <c r="B6" s="6" t="n">
+      <c r="B6" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
+      <c r="A7" s="1" t="n">
         <v>-0.03564688129</v>
       </c>
-      <c r="B7" s="6" t="n">
+      <c r="B7" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C7" s="5" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
+      <c r="A8" s="1" t="n">
         <v>-0.1518354392</v>
       </c>
-      <c r="B8" s="6" t="n">
+      <c r="B8" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C8" s="5" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
+      <c r="A9" s="1" t="n">
         <v>-0.07340816262</v>
       </c>
-      <c r="B9" s="6" t="n">
+      <c r="B9" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
+      <c r="A10" s="1" t="n">
         <v>-0.06167758706</v>
       </c>
-      <c r="B10" s="6" t="n">
+      <c r="B10" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="n">
+      <c r="A11" s="1" t="n">
         <v>0.005689432592</v>
       </c>
-      <c r="B11" s="6" t="n">
+      <c r="B11" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="n">
+      <c r="A12" s="1" t="n">
         <v>0.06635326621</v>
       </c>
-      <c r="B12" s="6" t="n">
+      <c r="B12" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="n">
+      <c r="A13" s="1" t="n">
         <v>0.06724702435</v>
       </c>
-      <c r="B13" s="6" t="n">
+      <c r="B13" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="n">
+      <c r="A14" s="1" t="n">
         <v>0.1786316323</v>
       </c>
-      <c r="B14" s="6" t="n">
+      <c r="B14" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="n">
+      <c r="A15" s="1" t="n">
         <v>0.0766314848</v>
       </c>
-      <c r="B15" s="6" t="n">
+      <c r="B15" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="n">
+      <c r="A16" s="1" t="n">
         <v>0.1915911253</v>
       </c>
-      <c r="B16" s="6" t="n">
+      <c r="B16" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C16" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="n">
+      <c r="A17" s="1" t="n">
         <v>0.1263467812</v>
       </c>
-      <c r="B17" s="6" t="n">
+      <c r="B17" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C17" s="5" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="n">
+      <c r="A18" s="1" t="n">
         <v>0.1069075417</v>
       </c>
-      <c r="B18" s="6" t="n">
+      <c r="B18" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="n">
+      <c r="A19" s="1" t="n">
         <v>0.1437750649</v>
       </c>
-      <c r="B19" s="6" t="n">
+      <c r="B19" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="n">
+      <c r="A20" s="1" t="n">
         <v>-0.02615070108</v>
       </c>
-      <c r="B20" s="6" t="n">
+      <c r="B20" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="n">
+      <c r="A21" s="1" t="n">
         <v>0.1119349312</v>
       </c>
-      <c r="B21" s="6" t="n">
+      <c r="B21" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="n">
+      <c r="A22" s="1" t="n">
         <v>-0.1126218009</v>
       </c>
-      <c r="B22" s="6" t="n">
+      <c r="B22" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="n">
+      <c r="A23" s="1" t="n">
         <v>-0.09698103351</v>
       </c>
-      <c r="B23" s="6" t="n">
+      <c r="B23" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="n">
+      <c r="A24" s="1" t="n">
         <v>0.006136311661</v>
       </c>
-      <c r="B24" s="6" t="n">
+      <c r="B24" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="n">
+      <c r="A25" s="1" t="n">
         <v>-0.02324598713</v>
       </c>
-      <c r="B25" s="6" t="n">
+      <c r="B25" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="n">
+      <c r="A26" s="1" t="n">
         <v>-0.05519784056</v>
       </c>
-      <c r="B26" s="6" t="n">
+      <c r="B26" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="n">
+      <c r="A27" s="1" t="n">
         <v>-0.0697214103</v>
       </c>
-      <c r="B27" s="6" t="n">
+      <c r="B27" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="n">
+      <c r="A28" s="1" t="n">
         <v>-0.138987666</v>
       </c>
-      <c r="B28" s="6" t="n">
+      <c r="B28" s="7" t="n">
         <v>45377</v>
       </c>
       <c r="C28" s="5" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="6"/>
+      <c r="B29" s="7"/>
       <c r="C29" s="5"/>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="6"/>
+      <c r="B30" s="7"/>
       <c r="C30" s="5"/>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="6"/>
+      <c r="B31" s="7"/>
       <c r="C31" s="5"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="6"/>
+      <c r="B32" s="7"/>
       <c r="C32" s="5"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="6"/>
+      <c r="B33" s="7"/>
       <c r="C33" s="5"/>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="6"/>
+      <c r="B34" s="7"/>
       <c r="C34" s="5"/>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="6"/>
+      <c r="B35" s="7"/>
       <c r="C35" s="5"/>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="6"/>
+      <c r="B36" s="7"/>
       <c r="C36" s="5"/>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="6"/>
+      <c r="B37" s="7"/>
       <c r="C37" s="5"/>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="6"/>
+      <c r="B38" s="7"/>
       <c r="C38" s="5"/>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="6"/>
+      <c r="B39" s="7"/>
       <c r="C39" s="5"/>
     </row>
   </sheetData>
@@ -2377,11 +2517,10 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <outlinePr summaryBelow="0"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D39"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34.51"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="35.75"/>
@@ -2389,548 +2528,548 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>100</v>
+        <v>113</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>102</v>
+        <v>115</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B2" s="7" t="n">
+      <c r="A2" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B2" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B3" s="7" t="n">
+      <c r="A3" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B3" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B4" s="7" t="n">
+      <c r="A4" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B4" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B5" s="7" t="n">
+      <c r="A5" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B5" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B6" s="7" t="n">
+      <c r="A6" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B6" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B7" s="7" t="n">
+      <c r="A7" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B7" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B8" s="7" t="n">
+      <c r="A8" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B8" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B9" s="7" t="n">
+      <c r="A9" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B9" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B10" s="7" t="n">
+      <c r="A10" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B10" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B11" s="7" t="n">
+      <c r="A11" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B11" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B12" s="7" t="n">
+      <c r="A12" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B12" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B13" s="7" t="n">
+      <c r="A13" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B13" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B14" s="7" t="n">
+      <c r="A14" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B14" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B15" s="7" t="n">
+      <c r="A15" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B15" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B16" s="7" t="n">
+      <c r="A16" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B16" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B17" s="7" t="n">
+      <c r="A17" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B17" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B18" s="7" t="n">
+      <c r="A18" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B18" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B19" s="7" t="n">
+      <c r="A19" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B19" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B20" s="7" t="n">
+      <c r="A20" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B20" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D20" s="5" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B21" s="7" t="n">
+      <c r="A21" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B21" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D21" s="5" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B22" s="7" t="n">
+      <c r="A22" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B22" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B23" s="7" t="n">
+      <c r="A23" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B23" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D23" s="5" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B24" s="7" t="n">
+      <c r="A24" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B24" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B25" s="7" t="n">
+      <c r="A25" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B25" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D25" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B26" s="7" t="n">
+      <c r="A26" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B26" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D26" s="5" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B27" s="7" t="n">
+      <c r="A27" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B27" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B28" s="7" t="n">
+      <c r="A28" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B28" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D28" s="5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B29" s="7" t="n">
+      <c r="A29" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B29" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B30" s="7" t="n">
+      <c r="A30" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B30" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B31" s="7" t="n">
+      <c r="A31" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B31" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B32" s="7" t="n">
+      <c r="A32" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B32" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D32" s="5" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B33" s="7" t="n">
+      <c r="A33" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B33" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D33" s="5" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B34" s="7" t="n">
+      <c r="A34" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B34" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D34" s="5" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B35" s="7" t="n">
+      <c r="A35" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B35" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B36" s="7" t="n">
+      <c r="A36" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B36" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B37" s="7" t="n">
+      <c r="A37" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B37" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B38" s="7" t="n">
+      <c r="A38" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B38" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D38" s="5" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="6" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B39" s="7" t="n">
+      <c r="A39" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B39" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>103</v>
+        <v>116</v>
       </c>
       <c r="D39" s="5" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correction métadonnées TMS4 et Dendromètre
</commit_message>
<xml_diff>
--- a/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
+++ b/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
@@ -191,7 +191,7 @@
     <t xml:space="preserve">Dendro_n°0</t>
   </si>
   <si>
-    <t xml:space="preserve">Dendro</t>
+    <t xml:space="preserve">Dendrometre</t>
   </si>
   <si>
     <t xml:space="preserve">identifiant_instrument (num_instrument)</t>
@@ -1547,6 +1547,12 @@
       <c r="D40" s="1" t="s">
         <v>53</v>
       </c>
+      <c r="E40" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="F40" s="1" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="n">
@@ -1558,8 +1564,14 @@
       <c r="C41" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="D41" s="0" t="s">
+      <c r="D41" s="1" t="s">
         <v>55</v>
+      </c>
+      <c r="E41" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="F41" s="1" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correction num_instrument des TMS4 et Dendromètre
</commit_message>
<xml_diff>
--- a/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
+++ b/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Instruments" sheetId="1" state="visible" r:id="rId3"/>
@@ -179,7 +179,7 @@
     <t xml:space="preserve">HOBO_n°38</t>
   </si>
   <si>
-    <t xml:space="preserve">TMS4_n°0</t>
+    <t xml:space="preserve">TMS4_95224601</t>
   </si>
   <si>
     <t xml:space="preserve">TOMST</t>
@@ -188,7 +188,7 @@
     <t xml:space="preserve">TMS4</t>
   </si>
   <si>
-    <t xml:space="preserve">Dendro_n°0</t>
+    <t xml:space="preserve">Dendro_92261195</t>
   </si>
   <si>
     <t xml:space="preserve">Dendrometre</t>
@@ -386,7 +386,7 @@
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -422,6 +422,12 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="0"/>
     </font>
     <font>
       <sz val="12"/>
@@ -480,7 +486,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -497,7 +503,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -505,7 +515,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1538,7 +1548,7 @@
       <c r="A40" s="1" t="n">
         <v>95224601</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" s="4" t="s">
         <v>51</v>
       </c>
       <c r="C40" s="1" t="s">
@@ -1558,7 +1568,7 @@
       <c r="A41" s="1" t="n">
         <v>92261195</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" s="4" t="s">
         <v>54</v>
       </c>
       <c r="C41" s="1" t="s">
@@ -1617,10 +1627,10 @@
       <c r="A2" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="4" t="n">
+      <c r="B2" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C2" s="5" t="s">
+      <c r="C2" s="6" t="s">
         <v>59</v>
       </c>
     </row>
@@ -1628,10 +1638,10 @@
       <c r="A3" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="4" t="n">
+      <c r="B3" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="6" t="s">
         <v>60</v>
       </c>
     </row>
@@ -1639,10 +1649,10 @@
       <c r="A4" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C4" s="5" t="s">
+      <c r="C4" s="6" t="s">
         <v>61</v>
       </c>
     </row>
@@ -1650,10 +1660,10 @@
       <c r="A5" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B5" s="4" t="n">
+      <c r="B5" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="6" t="s">
         <v>62</v>
       </c>
     </row>
@@ -1661,10 +1671,10 @@
       <c r="A6" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C6" s="5" t="s">
+      <c r="C6" s="6" t="s">
         <v>63</v>
       </c>
     </row>
@@ -1672,10 +1682,10 @@
       <c r="A7" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B7" s="4" t="n">
+      <c r="B7" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="6" t="s">
         <v>64</v>
       </c>
     </row>
@@ -1683,10 +1693,10 @@
       <c r="A8" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B8" s="4" t="n">
+      <c r="B8" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C8" s="5" t="s">
+      <c r="C8" s="6" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1694,10 +1704,10 @@
       <c r="A9" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="4" t="n">
+      <c r="B9" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="6" t="s">
         <v>66</v>
       </c>
     </row>
@@ -1705,10 +1715,10 @@
       <c r="A10" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="4" t="n">
+      <c r="B10" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C10" s="5" t="s">
+      <c r="C10" s="6" t="s">
         <v>67</v>
       </c>
     </row>
@@ -1716,10 +1726,10 @@
       <c r="A11" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B11" s="4" t="n">
+      <c r="B11" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="6" t="s">
         <v>68</v>
       </c>
     </row>
@@ -1727,10 +1737,10 @@
       <c r="A12" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B12" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C12" s="6" t="s">
         <v>69</v>
       </c>
     </row>
@@ -1738,10 +1748,10 @@
       <c r="A13" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B13" s="4" t="n">
+      <c r="B13" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="6" t="s">
         <v>70</v>
       </c>
     </row>
@@ -1749,10 +1759,10 @@
       <c r="A14" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B14" s="4" t="n">
+      <c r="B14" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C14" s="6" t="s">
         <v>71</v>
       </c>
     </row>
@@ -1760,10 +1770,10 @@
       <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="4" t="n">
+      <c r="B15" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C15" s="6" t="s">
         <v>72</v>
       </c>
     </row>
@@ -1771,10 +1781,10 @@
       <c r="A16" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="4" t="n">
+      <c r="B16" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C16" s="6" t="s">
         <v>73</v>
       </c>
     </row>
@@ -1782,10 +1792,10 @@
       <c r="A17" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B17" s="4" t="n">
+      <c r="B17" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C17" s="5" t="s">
+      <c r="C17" s="6" t="s">
         <v>74</v>
       </c>
     </row>
@@ -1793,10 +1803,10 @@
       <c r="A18" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B18" s="4" t="n">
+      <c r="B18" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="C18" s="6" t="s">
         <v>75</v>
       </c>
     </row>
@@ -1804,10 +1814,10 @@
       <c r="A19" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B19" s="4" t="n">
+      <c r="B19" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C19" s="5" t="s">
+      <c r="C19" s="6" t="s">
         <v>76</v>
       </c>
     </row>
@@ -1815,10 +1825,10 @@
       <c r="A20" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B20" s="4" t="n">
+      <c r="B20" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C20" s="5" t="s">
+      <c r="C20" s="6" t="s">
         <v>77</v>
       </c>
     </row>
@@ -1826,10 +1836,10 @@
       <c r="A21" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B21" s="4" t="n">
+      <c r="B21" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="C21" s="6" t="s">
         <v>78</v>
       </c>
     </row>
@@ -1837,10 +1847,10 @@
       <c r="A22" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="4" t="n">
+      <c r="B22" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C22" s="5" t="s">
+      <c r="C22" s="6" t="s">
         <v>79</v>
       </c>
     </row>
@@ -1848,10 +1858,10 @@
       <c r="A23" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B23" s="4" t="n">
+      <c r="B23" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C23" s="5" t="s">
+      <c r="C23" s="6" t="s">
         <v>80</v>
       </c>
     </row>
@@ -1859,10 +1869,10 @@
       <c r="A24" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="4" t="n">
+      <c r="B24" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C24" s="5" t="s">
+      <c r="C24" s="6" t="s">
         <v>81</v>
       </c>
     </row>
@@ -1870,10 +1880,10 @@
       <c r="A25" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B25" s="4" t="n">
+      <c r="B25" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C25" s="5" t="s">
+      <c r="C25" s="6" t="s">
         <v>82</v>
       </c>
     </row>
@@ -1881,10 +1891,10 @@
       <c r="A26" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B26" s="4" t="n">
+      <c r="B26" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C26" s="5" t="s">
+      <c r="C26" s="6" t="s">
         <v>83</v>
       </c>
     </row>
@@ -1892,10 +1902,10 @@
       <c r="A27" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B27" s="4" t="n">
+      <c r="B27" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C27" s="5" t="s">
+      <c r="C27" s="6" t="s">
         <v>84</v>
       </c>
     </row>
@@ -1903,10 +1913,10 @@
       <c r="A28" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B28" s="4" t="n">
+      <c r="B28" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C28" s="5" t="s">
+      <c r="C28" s="6" t="s">
         <v>85</v>
       </c>
     </row>
@@ -1914,10 +1924,10 @@
       <c r="A29" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B29" s="4" t="n">
+      <c r="B29" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C29" s="5" t="s">
+      <c r="C29" s="6" t="s">
         <v>86</v>
       </c>
     </row>
@@ -1925,10 +1935,10 @@
       <c r="A30" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B30" s="4" t="n">
+      <c r="B30" s="5" t="n">
         <v>46098</v>
       </c>
-      <c r="C30" s="5" t="s">
+      <c r="C30" s="6" t="s">
         <v>87</v>
       </c>
     </row>
@@ -1936,10 +1946,10 @@
       <c r="A31" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B31" s="4" t="n">
+      <c r="B31" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C31" s="5" t="s">
+      <c r="C31" s="6" t="s">
         <v>88</v>
       </c>
     </row>
@@ -1947,10 +1957,10 @@
       <c r="A32" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B32" s="4" t="n">
+      <c r="B32" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C32" s="5" t="s">
+      <c r="C32" s="6" t="s">
         <v>89</v>
       </c>
     </row>
@@ -1958,10 +1968,10 @@
       <c r="A33" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B33" s="4" t="n">
+      <c r="B33" s="5" t="n">
         <v>46098</v>
       </c>
-      <c r="C33" s="5" t="s">
+      <c r="C33" s="6" t="s">
         <v>90</v>
       </c>
     </row>
@@ -1969,10 +1979,10 @@
       <c r="A34" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B34" s="4" t="n">
+      <c r="B34" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C34" s="5" t="s">
+      <c r="C34" s="6" t="s">
         <v>91</v>
       </c>
     </row>
@@ -1980,8 +1990,8 @@
       <c r="A35" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B35" s="4"/>
-      <c r="C35" s="5" t="s">
+      <c r="B35" s="5"/>
+      <c r="C35" s="6" t="s">
         <v>92</v>
       </c>
     </row>
@@ -1989,8 +1999,8 @@
       <c r="A36" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B36" s="4"/>
-      <c r="C36" s="5" t="s">
+      <c r="B36" s="5"/>
+      <c r="C36" s="6" t="s">
         <v>93</v>
       </c>
     </row>
@@ -1998,10 +2008,10 @@
       <c r="A37" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B37" s="4" t="n">
+      <c r="B37" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C37" s="5" t="s">
+      <c r="C37" s="6" t="s">
         <v>94</v>
       </c>
     </row>
@@ -2009,8 +2019,8 @@
       <c r="A38" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B38" s="4"/>
-      <c r="C38" s="5" t="s">
+      <c r="B38" s="5"/>
+      <c r="C38" s="6" t="s">
         <v>95</v>
       </c>
     </row>
@@ -2018,76 +2028,76 @@
       <c r="A39" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B39" s="4" t="n">
+      <c r="B39" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C39" s="5" t="s">
+      <c r="C39" s="6" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="s">
+      <c r="A40" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B40" s="6" t="s">
+      <c r="B40" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="C40" s="5" t="s">
+      <c r="C40" s="6" t="s">
         <v>98</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5" t="s">
+      <c r="A41" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B41" s="6" t="s">
+      <c r="B41" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="C41" s="5" t="s">
+      <c r="C41" s="6" t="s">
         <v>99</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="s">
+      <c r="A42" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="C42" s="5" t="s">
+      <c r="C42" s="6" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="5" t="s">
+      <c r="A43" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B43" s="6" t="s">
+      <c r="B43" s="7" t="s">
         <v>97</v>
       </c>
-      <c r="C43" s="5" t="s">
+      <c r="C43" s="6" t="s">
         <v>101</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="1" t="s">
+      <c r="A44" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B44" s="6" t="s">
+      <c r="B44" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="C44" s="5" t="s">
+      <c r="C44" s="6" t="s">
         <v>103</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="1" t="s">
+      <c r="A45" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B45" s="6" t="s">
+      <c r="B45" s="7" t="s">
         <v>102</v>
       </c>
-      <c r="C45" s="5" t="s">
+      <c r="C45" s="6" t="s">
         <v>104</v>
       </c>
     </row>
@@ -2135,8 +2145,8 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2178,10 +2188,10 @@
       <c r="A2" s="1" t="n">
         <v>-0.09653415444</v>
       </c>
-      <c r="B2" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C2" s="5" t="s">
+      <c r="B2" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>60</v>
       </c>
     </row>
@@ -2189,10 +2199,10 @@
       <c r="A3" s="1" t="n">
         <v>-0.08044650796</v>
       </c>
-      <c r="B3" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C3" s="5" t="s">
+      <c r="B3" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C3" s="6" t="s">
         <v>61</v>
       </c>
     </row>
@@ -2200,10 +2210,10 @@
       <c r="A4" s="1" t="n">
         <v>0.05317033367</v>
       </c>
-      <c r="B4" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C4" s="5" t="s">
+      <c r="B4" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>62</v>
       </c>
     </row>
@@ -2211,10 +2221,10 @@
       <c r="A5" s="1" t="n">
         <v>-0.0570970766</v>
       </c>
-      <c r="B5" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C5" s="5" t="s">
+      <c r="B5" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C5" s="6" t="s">
         <v>63</v>
       </c>
     </row>
@@ -2222,10 +2232,10 @@
       <c r="A6" s="1" t="n">
         <v>-0.05486268126</v>
       </c>
-      <c r="B6" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C6" s="5" t="s">
+      <c r="B6" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>64</v>
       </c>
     </row>
@@ -2233,10 +2243,10 @@
       <c r="A7" s="1" t="n">
         <v>-0.03564688129</v>
       </c>
-      <c r="B7" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C7" s="5" t="s">
+      <c r="B7" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C7" s="6" t="s">
         <v>65</v>
       </c>
     </row>
@@ -2244,10 +2254,10 @@
       <c r="A8" s="1" t="n">
         <v>-0.1518354392</v>
       </c>
-      <c r="B8" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C8" s="5" t="s">
+      <c r="B8" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C8" s="6" t="s">
         <v>67</v>
       </c>
     </row>
@@ -2255,10 +2265,10 @@
       <c r="A9" s="1" t="n">
         <v>-0.07340816262</v>
       </c>
-      <c r="B9" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C9" s="5" t="s">
+      <c r="B9" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>69</v>
       </c>
     </row>
@@ -2266,10 +2276,10 @@
       <c r="A10" s="1" t="n">
         <v>-0.06167758706</v>
       </c>
-      <c r="B10" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C10" s="5" t="s">
+      <c r="B10" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C10" s="6" t="s">
         <v>70</v>
       </c>
     </row>
@@ -2277,10 +2287,10 @@
       <c r="A11" s="1" t="n">
         <v>0.005689432592</v>
       </c>
-      <c r="B11" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C11" s="5" t="s">
+      <c r="B11" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C11" s="6" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2288,10 +2298,10 @@
       <c r="A12" s="1" t="n">
         <v>0.06635326621</v>
       </c>
-      <c r="B12" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C12" s="5" t="s">
+      <c r="B12" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>72</v>
       </c>
     </row>
@@ -2299,10 +2309,10 @@
       <c r="A13" s="1" t="n">
         <v>0.06724702435</v>
       </c>
-      <c r="B13" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C13" s="5" t="s">
+      <c r="B13" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C13" s="6" t="s">
         <v>73</v>
       </c>
     </row>
@@ -2310,10 +2320,10 @@
       <c r="A14" s="1" t="n">
         <v>0.1786316323</v>
       </c>
-      <c r="B14" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C14" s="5" t="s">
+      <c r="B14" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>74</v>
       </c>
     </row>
@@ -2321,10 +2331,10 @@
       <c r="A15" s="1" t="n">
         <v>0.0766314848</v>
       </c>
-      <c r="B15" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C15" s="5" t="s">
+      <c r="B15" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C15" s="6" t="s">
         <v>75</v>
       </c>
     </row>
@@ -2332,10 +2342,10 @@
       <c r="A16" s="1" t="n">
         <v>0.1915911253</v>
       </c>
-      <c r="B16" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C16" s="5" t="s">
+      <c r="B16" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C16" s="6" t="s">
         <v>76</v>
       </c>
     </row>
@@ -2343,10 +2353,10 @@
       <c r="A17" s="1" t="n">
         <v>0.1263467812</v>
       </c>
-      <c r="B17" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C17" s="5" t="s">
+      <c r="B17" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>77</v>
       </c>
     </row>
@@ -2354,10 +2364,10 @@
       <c r="A18" s="1" t="n">
         <v>0.1069075417</v>
       </c>
-      <c r="B18" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C18" s="5" t="s">
+      <c r="B18" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C18" s="6" t="s">
         <v>78</v>
       </c>
     </row>
@@ -2365,10 +2375,10 @@
       <c r="A19" s="1" t="n">
         <v>0.1437750649</v>
       </c>
-      <c r="B19" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C19" s="5" t="s">
+      <c r="B19" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C19" s="6" t="s">
         <v>79</v>
       </c>
     </row>
@@ -2376,10 +2386,10 @@
       <c r="A20" s="1" t="n">
         <v>-0.02615070108</v>
       </c>
-      <c r="B20" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C20" s="5" t="s">
+      <c r="B20" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C20" s="6" t="s">
         <v>80</v>
       </c>
     </row>
@@ -2387,10 +2397,10 @@
       <c r="A21" s="1" t="n">
         <v>0.1119349312</v>
       </c>
-      <c r="B21" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C21" s="5" t="s">
+      <c r="B21" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C21" s="6" t="s">
         <v>81</v>
       </c>
     </row>
@@ -2398,10 +2408,10 @@
       <c r="A22" s="1" t="n">
         <v>-0.1126218009</v>
       </c>
-      <c r="B22" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C22" s="5" t="s">
+      <c r="B22" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>82</v>
       </c>
     </row>
@@ -2409,10 +2419,10 @@
       <c r="A23" s="1" t="n">
         <v>-0.09698103351</v>
       </c>
-      <c r="B23" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C23" s="5" t="s">
+      <c r="B23" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C23" s="6" t="s">
         <v>83</v>
       </c>
     </row>
@@ -2420,10 +2430,10 @@
       <c r="A24" s="1" t="n">
         <v>0.006136311661</v>
       </c>
-      <c r="B24" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C24" s="5" t="s">
+      <c r="B24" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C24" s="6" t="s">
         <v>84</v>
       </c>
     </row>
@@ -2431,10 +2441,10 @@
       <c r="A25" s="1" t="n">
         <v>-0.02324598713</v>
       </c>
-      <c r="B25" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C25" s="5" t="s">
+      <c r="B25" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C25" s="6" t="s">
         <v>86</v>
       </c>
     </row>
@@ -2442,10 +2452,10 @@
       <c r="A26" s="1" t="n">
         <v>-0.05519784056</v>
       </c>
-      <c r="B26" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C26" s="5" t="s">
+      <c r="B26" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C26" s="6" t="s">
         <v>88</v>
       </c>
     </row>
@@ -2453,10 +2463,10 @@
       <c r="A27" s="1" t="n">
         <v>-0.0697214103</v>
       </c>
-      <c r="B27" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C27" s="5" t="s">
+      <c r="B27" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C27" s="6" t="s">
         <v>89</v>
       </c>
     </row>
@@ -2464,56 +2474,56 @@
       <c r="A28" s="1" t="n">
         <v>-0.138987666</v>
       </c>
-      <c r="B28" s="7" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C28" s="5" t="s">
+      <c r="B28" s="8" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C28" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="7"/>
-      <c r="C29" s="5"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="6"/>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="7"/>
-      <c r="C30" s="5"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="6"/>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="7"/>
-      <c r="C31" s="5"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="6"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="7"/>
-      <c r="C32" s="5"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="6"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="7"/>
-      <c r="C33" s="5"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="6"/>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="7"/>
-      <c r="C34" s="5"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="6"/>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="7"/>
-      <c r="C35" s="5"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="6"/>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="7"/>
-      <c r="C36" s="5"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="6"/>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="7"/>
-      <c r="C37" s="5"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="6"/>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="7"/>
-      <c r="C38" s="5"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="6"/>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="7"/>
-      <c r="C39" s="5"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="6"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2553,534 +2563,534 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B2" s="8" t="n">
+      <c r="A2" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B2" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="6" t="s">
         <v>59</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B3" s="8" t="n">
+      <c r="A3" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B3" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="6" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B4" s="8" t="n">
+      <c r="A4" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B4" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="6" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B5" s="8" t="n">
+      <c r="A5" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B5" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="6" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B6" s="8" t="n">
+      <c r="A6" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B6" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="6" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B7" s="8" t="n">
+      <c r="A7" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B7" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="6" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B8" s="8" t="n">
+      <c r="A8" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B8" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="6" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B9" s="8" t="n">
+      <c r="A9" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B9" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="6" t="s">
         <v>66</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B10" s="8" t="n">
+      <c r="A10" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B10" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="6" t="s">
         <v>67</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B11" s="8" t="n">
+      <c r="A11" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B11" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="6" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B12" s="8" t="n">
+      <c r="A12" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B12" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D12" s="6" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B13" s="8" t="n">
+      <c r="A13" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B13" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>70</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B14" s="8" t="n">
+      <c r="A14" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B14" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>71</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B15" s="8" t="n">
+      <c r="A15" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B15" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="D15" s="6" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B16" s="8" t="n">
+      <c r="A16" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B16" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="D16" s="6" t="s">
         <v>73</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B17" s="8" t="n">
+      <c r="A17" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B17" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D17" s="6" t="s">
         <v>74</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B18" s="8" t="n">
+      <c r="A18" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B18" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="D18" s="6" t="s">
         <v>75</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B19" s="8" t="n">
+      <c r="A19" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B19" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D19" s="6" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B20" s="8" t="n">
+      <c r="A20" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B20" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="D20" s="6" t="s">
         <v>77</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B21" s="8" t="n">
+      <c r="A21" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B21" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D21" s="5" t="s">
+      <c r="D21" s="6" t="s">
         <v>78</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B22" s="8" t="n">
+      <c r="A22" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B22" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="D22" s="6" t="s">
         <v>79</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B23" s="8" t="n">
+      <c r="A23" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B23" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="6" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B24" s="8" t="n">
+      <c r="A24" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B24" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="6" t="s">
         <v>81</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B25" s="8" t="n">
+      <c r="A25" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B25" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="D25" s="6" t="s">
         <v>82</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B26" s="8" t="n">
+      <c r="A26" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B26" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D26" s="6" t="s">
         <v>83</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B27" s="8" t="n">
+      <c r="A27" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B27" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D27" s="6" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B28" s="8" t="n">
+      <c r="A28" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B28" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="D28" s="6" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B29" s="8" t="n">
+      <c r="A29" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B29" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D29" s="6" t="s">
         <v>86</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B30" s="8" t="n">
+      <c r="A30" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B30" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="6" t="s">
         <v>87</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B31" s="8" t="n">
+      <c r="A31" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B31" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="D31" s="6" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B32" s="8" t="n">
+      <c r="A32" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B32" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="D32" s="6" t="s">
         <v>89</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B33" s="8" t="n">
+      <c r="A33" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B33" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="D33" s="6" t="s">
         <v>90</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B34" s="8" t="n">
+      <c r="A34" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B34" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="D34" s="6" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B35" s="8" t="n">
+      <c r="A35" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B35" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D35" s="6" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B36" s="8" t="n">
+      <c r="A36" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B36" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D36" s="6" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B37" s="8" t="n">
+      <c r="A37" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B37" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="D37" s="6" t="s">
         <v>94</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B38" s="8" t="n">
+      <c r="A38" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B38" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="D38" s="6" t="s">
         <v>95</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="7" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B39" s="8" t="n">
+      <c r="A39" s="8" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B39" s="9" t="n">
         <v>45377</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>116</v>
       </c>
-      <c r="D39" s="5" t="s">
+      <c r="D39" s="6" t="s">
         <v>96</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Intégration complète corrigée des instruments TOMST (TMS4, Dendromètre et Thermologger)
</commit_message>
<xml_diff>
--- a/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
+++ b/Base_de_donnees/Fichiers_metadonnees/Metadonnees_instruments_capteurs.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Instruments" sheetId="1" state="visible" r:id="rId3"/>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="350" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="351" uniqueCount="118">
   <si>
     <t xml:space="preserve">numéro_serie</t>
   </si>
@@ -201,6 +201,9 @@
   </si>
   <si>
     <t xml:space="preserve">description (unique)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">num_colonne</t>
   </si>
   <si>
     <t xml:space="preserve">capteur de température du HOBO n°01</t>
@@ -386,7 +389,7 @@
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yy"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -422,12 +425,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Arial"/>
-      <family val="0"/>
     </font>
     <font>
       <sz val="12"/>
@@ -486,7 +483,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -503,19 +500,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1606,7 +1599,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.88"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="25.38"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="43.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="85.38"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="20.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="21.38"/>
   </cols>
   <sheetData>
@@ -1620,7 +1613,9 @@
       <c r="C1" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D1" s="2"/>
+      <c r="D1" s="2" t="s">
+        <v>59</v>
+      </c>
       <c r="E1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1630,8 +1625,11 @@
       <c r="B2" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>59</v>
+      <c r="C2" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1641,8 +1639,11 @@
       <c r="B3" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C3" s="6" t="s">
-        <v>60</v>
+      <c r="C3" s="4" t="s">
+        <v>61</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1652,8 +1653,11 @@
       <c r="B4" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C4" s="6" t="s">
-        <v>61</v>
+      <c r="C4" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1663,8 +1667,11 @@
       <c r="B5" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>62</v>
+      <c r="C5" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1674,8 +1681,11 @@
       <c r="B6" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C6" s="6" t="s">
-        <v>63</v>
+      <c r="C6" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1685,8 +1695,11 @@
       <c r="B7" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>64</v>
+      <c r="C7" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1696,8 +1709,11 @@
       <c r="B8" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>65</v>
+      <c r="C8" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1707,8 +1723,11 @@
       <c r="B9" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>66</v>
+      <c r="C9" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1718,8 +1737,11 @@
       <c r="B10" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>67</v>
+      <c r="C10" s="4" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1729,8 +1751,11 @@
       <c r="B11" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>68</v>
+      <c r="C11" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D11" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1740,8 +1765,11 @@
       <c r="B12" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>69</v>
+      <c r="C12" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1751,8 +1779,11 @@
       <c r="B13" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C13" s="6" t="s">
-        <v>70</v>
+      <c r="C13" s="4" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1762,8 +1793,11 @@
       <c r="B14" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C14" s="6" t="s">
-        <v>71</v>
+      <c r="C14" s="4" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1773,8 +1807,11 @@
       <c r="B15" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C15" s="6" t="s">
-        <v>72</v>
+      <c r="C15" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1784,8 +1821,11 @@
       <c r="B16" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C16" s="6" t="s">
-        <v>73</v>
+      <c r="C16" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1795,8 +1835,11 @@
       <c r="B17" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>74</v>
+      <c r="C17" s="4" t="s">
+        <v>75</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1806,8 +1849,11 @@
       <c r="B18" s="5" t="n">
         <v>45412</v>
       </c>
-      <c r="C18" s="6" t="s">
-        <v>75</v>
+      <c r="C18" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="D18" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1817,8 +1863,11 @@
       <c r="B19" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C19" s="6" t="s">
-        <v>76</v>
+      <c r="C19" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D19" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1828,8 +1877,11 @@
       <c r="B20" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C20" s="6" t="s">
-        <v>77</v>
+      <c r="C20" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1839,8 +1891,11 @@
       <c r="B21" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C21" s="6" t="s">
-        <v>78</v>
+      <c r="C21" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1850,8 +1905,11 @@
       <c r="B22" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C22" s="6" t="s">
-        <v>79</v>
+      <c r="C22" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="D22" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1861,8 +1919,11 @@
       <c r="B23" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C23" s="6" t="s">
-        <v>80</v>
+      <c r="C23" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D23" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1872,8 +1933,11 @@
       <c r="B24" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C24" s="6" t="s">
-        <v>81</v>
+      <c r="C24" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1883,8 +1947,11 @@
       <c r="B25" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C25" s="6" t="s">
-        <v>82</v>
+      <c r="C25" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1894,8 +1961,11 @@
       <c r="B26" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C26" s="6" t="s">
-        <v>83</v>
+      <c r="C26" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1905,8 +1975,11 @@
       <c r="B27" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C27" s="6" t="s">
-        <v>84</v>
+      <c r="C27" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="D27" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1916,8 +1989,11 @@
       <c r="B28" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C28" s="6" t="s">
-        <v>85</v>
+      <c r="C28" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1927,8 +2003,11 @@
       <c r="B29" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C29" s="6" t="s">
-        <v>86</v>
+      <c r="C29" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1938,8 +2017,11 @@
       <c r="B30" s="5" t="n">
         <v>46098</v>
       </c>
-      <c r="C30" s="6" t="s">
-        <v>87</v>
+      <c r="C30" s="4" t="s">
+        <v>88</v>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1949,8 +2031,11 @@
       <c r="B31" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C31" s="6" t="s">
-        <v>88</v>
+      <c r="C31" s="4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1960,8 +2045,11 @@
       <c r="B32" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C32" s="6" t="s">
-        <v>89</v>
+      <c r="C32" s="4" t="s">
+        <v>90</v>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1971,8 +2059,11 @@
       <c r="B33" s="5" t="n">
         <v>46098</v>
       </c>
-      <c r="C33" s="6" t="s">
-        <v>90</v>
+      <c r="C33" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1982,8 +2073,11 @@
       <c r="B34" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C34" s="6" t="s">
-        <v>91</v>
+      <c r="C34" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1991,8 +2085,11 @@
         <v>45</v>
       </c>
       <c r="B35" s="5"/>
-      <c r="C35" s="6" t="s">
-        <v>92</v>
+      <c r="C35" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2000,8 +2097,11 @@
         <v>47</v>
       </c>
       <c r="B36" s="5"/>
-      <c r="C36" s="6" t="s">
-        <v>93</v>
+      <c r="C36" s="4" t="s">
+        <v>94</v>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2011,8 +2111,11 @@
       <c r="B37" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C37" s="6" t="s">
-        <v>94</v>
+      <c r="C37" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2020,8 +2123,11 @@
         <v>49</v>
       </c>
       <c r="B38" s="5"/>
-      <c r="C38" s="6" t="s">
-        <v>95</v>
+      <c r="C38" s="4" t="s">
+        <v>96</v>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2031,74 +2137,95 @@
       <c r="B39" s="5" t="n">
         <v>45451</v>
       </c>
-      <c r="C39" s="6" t="s">
-        <v>96</v>
+      <c r="C39" s="4" t="s">
+        <v>97</v>
+      </c>
+      <c r="D39" s="1" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B40" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C40" s="6" t="s">
+      <c r="B40" s="6" t="s">
         <v>98</v>
+      </c>
+      <c r="C40" s="4" t="s">
+        <v>99</v>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B41" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C41" s="6" t="s">
-        <v>99</v>
+      <c r="B41" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C41" s="4" t="s">
+        <v>100</v>
+      </c>
+      <c r="D41" s="1" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B42" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C42" s="6" t="s">
-        <v>100</v>
+      <c r="B42" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C42" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="D42" s="1" t="n">
+        <v>6</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="B43" s="7" t="s">
-        <v>97</v>
-      </c>
-      <c r="C43" s="6" t="s">
-        <v>101</v>
+      <c r="B43" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="C43" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>7</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B44" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="C44" s="6" t="s">
+      <c r="B44" s="6" t="s">
         <v>103</v>
+      </c>
+      <c r="C44" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="D44" s="1" t="n">
+        <v>4</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B45" s="7" t="s">
-        <v>102</v>
-      </c>
-      <c r="C45" s="6" t="s">
-        <v>104</v>
+      <c r="B45" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="C45" s="4" t="s">
+        <v>105</v>
+      </c>
+      <c r="D45" s="1" t="n">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -2129,24 +2256,24 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2175,355 +2302,355 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="1" t="n">
         <v>-0.09653415444</v>
       </c>
-      <c r="B2" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>60</v>
+      <c r="B2" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="1" t="n">
         <v>-0.08044650796</v>
       </c>
-      <c r="B3" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C3" s="6" t="s">
-        <v>61</v>
+      <c r="B3" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C3" s="4" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="1" t="n">
         <v>0.05317033367</v>
       </c>
-      <c r="B4" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C4" s="6" t="s">
-        <v>62</v>
+      <c r="B4" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="1" t="n">
         <v>-0.0570970766</v>
       </c>
-      <c r="B5" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C5" s="6" t="s">
-        <v>63</v>
+      <c r="B5" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="1" t="n">
         <v>-0.05486268126</v>
       </c>
-      <c r="B6" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C6" s="6" t="s">
-        <v>64</v>
+      <c r="B6" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="1" t="n">
         <v>-0.03564688129</v>
       </c>
-      <c r="B7" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>65</v>
+      <c r="B7" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="1" t="n">
         <v>-0.1518354392</v>
       </c>
-      <c r="B8" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>67</v>
+      <c r="B8" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="1" t="n">
         <v>-0.07340816262</v>
       </c>
-      <c r="B9" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>69</v>
+      <c r="B9" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="1" t="n">
         <v>-0.06167758706</v>
       </c>
-      <c r="B10" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>70</v>
+      <c r="B10" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="1" t="n">
         <v>0.005689432592</v>
       </c>
-      <c r="B11" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C11" s="6" t="s">
-        <v>71</v>
+      <c r="B11" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="1" t="n">
         <v>0.06635326621</v>
       </c>
-      <c r="B12" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C12" s="6" t="s">
-        <v>72</v>
+      <c r="B12" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="1" t="n">
         <v>0.06724702435</v>
       </c>
-      <c r="B13" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>73</v>
+      <c r="B13" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="1" t="n">
         <v>0.1786316323</v>
       </c>
-      <c r="B14" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>74</v>
+      <c r="B14" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="1" t="n">
         <v>0.0766314848</v>
       </c>
-      <c r="B15" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C15" s="6" t="s">
-        <v>75</v>
+      <c r="B15" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="1" t="n">
         <v>0.1915911253</v>
       </c>
-      <c r="B16" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C16" s="6" t="s">
-        <v>76</v>
+      <c r="B16" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="1" t="n">
         <v>0.1263467812</v>
       </c>
-      <c r="B17" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C17" s="6" t="s">
-        <v>77</v>
+      <c r="B17" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="1" t="n">
         <v>0.1069075417</v>
       </c>
-      <c r="B18" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C18" s="6" t="s">
-        <v>78</v>
+      <c r="B18" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="1" t="n">
         <v>0.1437750649</v>
       </c>
-      <c r="B19" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C19" s="6" t="s">
-        <v>79</v>
+      <c r="B19" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="1" t="n">
         <v>-0.02615070108</v>
       </c>
-      <c r="B20" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C20" s="6" t="s">
-        <v>80</v>
+      <c r="B20" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="1" t="n">
         <v>0.1119349312</v>
       </c>
-      <c r="B21" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C21" s="6" t="s">
-        <v>81</v>
+      <c r="B21" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="1" t="n">
         <v>-0.1126218009</v>
       </c>
-      <c r="B22" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C22" s="6" t="s">
-        <v>82</v>
+      <c r="B22" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="1" t="n">
         <v>-0.09698103351</v>
       </c>
-      <c r="B23" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C23" s="6" t="s">
-        <v>83</v>
+      <c r="B23" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="1" t="n">
         <v>0.006136311661</v>
       </c>
-      <c r="B24" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C24" s="6" t="s">
-        <v>84</v>
+      <c r="B24" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="1" t="n">
         <v>-0.02324598713</v>
       </c>
-      <c r="B25" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C25" s="6" t="s">
-        <v>86</v>
+      <c r="B25" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="1" t="n">
         <v>-0.05519784056</v>
       </c>
-      <c r="B26" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C26" s="6" t="s">
-        <v>88</v>
+      <c r="B26" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="1" t="n">
         <v>-0.0697214103</v>
       </c>
-      <c r="B27" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C27" s="6" t="s">
-        <v>89</v>
+      <c r="B27" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="1" t="n">
         <v>-0.138987666</v>
       </c>
-      <c r="B28" s="8" t="n">
-        <v>45377</v>
-      </c>
-      <c r="C28" s="6" t="s">
-        <v>94</v>
+      <c r="B28" s="7" t="n">
+        <v>45377</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B29" s="8"/>
-      <c r="C29" s="6"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="4"/>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B30" s="8"/>
-      <c r="C30" s="6"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="4"/>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B31" s="8"/>
-      <c r="C31" s="6"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="4"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="8"/>
-      <c r="C32" s="6"/>
+      <c r="B32" s="7"/>
+      <c r="C32" s="4"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B33" s="8"/>
-      <c r="C33" s="6"/>
+      <c r="B33" s="7"/>
+      <c r="C33" s="4"/>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B34" s="8"/>
-      <c r="C34" s="6"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="4"/>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B35" s="8"/>
-      <c r="C35" s="6"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="4"/>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B36" s="8"/>
-      <c r="C36" s="6"/>
+      <c r="B36" s="7"/>
+      <c r="C36" s="4"/>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B37" s="8"/>
-      <c r="C37" s="6"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="4"/>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B38" s="8"/>
-      <c r="C38" s="6"/>
+      <c r="B38" s="7"/>
+      <c r="C38" s="4"/>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B39" s="8"/>
-      <c r="C39" s="6"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="4"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2550,548 +2677,548 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>6</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B2" s="9" t="n">
+      <c r="A2" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B2" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>59</v>
+        <v>117</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B3" s="9" t="n">
+      <c r="A3" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B3" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D3" s="6" t="s">
-        <v>60</v>
+        <v>117</v>
+      </c>
+      <c r="D3" s="4" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B4" s="9" t="n">
+      <c r="A4" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B4" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>61</v>
+        <v>117</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B5" s="9" t="n">
+      <c r="A5" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B5" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D5" s="6" t="s">
-        <v>62</v>
+        <v>117</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B6" s="9" t="n">
+      <c r="A6" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B6" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>63</v>
+        <v>117</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B7" s="9" t="n">
+      <c r="A7" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B7" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D7" s="6" t="s">
-        <v>64</v>
+        <v>117</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B8" s="9" t="n">
+      <c r="A8" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B8" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>65</v>
+        <v>117</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B9" s="9" t="n">
+      <c r="A9" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B9" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D9" s="6" t="s">
-        <v>66</v>
+        <v>117</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B10" s="9" t="n">
+      <c r="A10" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B10" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>67</v>
+        <v>117</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B11" s="9" t="n">
+      <c r="A11" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B11" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D11" s="6" t="s">
-        <v>68</v>
+        <v>117</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B12" s="9" t="n">
+      <c r="A12" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B12" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>69</v>
+        <v>117</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B13" s="9" t="n">
+      <c r="A13" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B13" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D13" s="6" t="s">
-        <v>70</v>
+        <v>117</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B14" s="9" t="n">
+      <c r="A14" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B14" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D14" s="6" t="s">
-        <v>71</v>
+        <v>117</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B15" s="9" t="n">
+      <c r="A15" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B15" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>72</v>
+        <v>117</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>73</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B16" s="9" t="n">
+      <c r="A16" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B16" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D16" s="6" t="s">
-        <v>73</v>
+        <v>117</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B17" s="9" t="n">
+      <c r="A17" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B17" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D17" s="6" t="s">
-        <v>74</v>
+        <v>117</v>
+      </c>
+      <c r="D17" s="4" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B18" s="9" t="n">
+      <c r="A18" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B18" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D18" s="6" t="s">
-        <v>75</v>
+        <v>117</v>
+      </c>
+      <c r="D18" s="4" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B19" s="9" t="n">
+      <c r="A19" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B19" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D19" s="6" t="s">
-        <v>76</v>
+        <v>117</v>
+      </c>
+      <c r="D19" s="4" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B20" s="9" t="n">
+      <c r="A20" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B20" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D20" s="6" t="s">
-        <v>77</v>
+        <v>117</v>
+      </c>
+      <c r="D20" s="4" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B21" s="9" t="n">
+      <c r="A21" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B21" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>78</v>
+        <v>117</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B22" s="9" t="n">
+      <c r="A22" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B22" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>79</v>
+        <v>117</v>
+      </c>
+      <c r="D22" s="4" t="s">
+        <v>80</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B23" s="9" t="n">
+      <c r="A23" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B23" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D23" s="6" t="s">
-        <v>80</v>
+        <v>117</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>81</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B24" s="9" t="n">
+      <c r="A24" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B24" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D24" s="6" t="s">
-        <v>81</v>
+        <v>117</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>82</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B25" s="9" t="n">
+      <c r="A25" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B25" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D25" s="6" t="s">
-        <v>82</v>
+        <v>117</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B26" s="9" t="n">
+      <c r="A26" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B26" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D26" s="6" t="s">
-        <v>83</v>
+        <v>117</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B27" s="9" t="n">
+      <c r="A27" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B27" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D27" s="6" t="s">
-        <v>84</v>
+        <v>117</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B28" s="9" t="n">
+      <c r="A28" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B28" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D28" s="6" t="s">
-        <v>85</v>
+        <v>117</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>86</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B29" s="9" t="n">
+      <c r="A29" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B29" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D29" s="6" t="s">
-        <v>86</v>
+        <v>117</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>87</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B30" s="9" t="n">
+      <c r="A30" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B30" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D30" s="6" t="s">
-        <v>87</v>
+        <v>117</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>88</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B31" s="9" t="n">
+      <c r="A31" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B31" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D31" s="6" t="s">
-        <v>88</v>
+        <v>117</v>
+      </c>
+      <c r="D31" s="4" t="s">
+        <v>89</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B32" s="9" t="n">
+      <c r="A32" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B32" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D32" s="6" t="s">
-        <v>89</v>
+        <v>117</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B33" s="9" t="n">
+      <c r="A33" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B33" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D33" s="6" t="s">
-        <v>90</v>
+        <v>117</v>
+      </c>
+      <c r="D33" s="4" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B34" s="9" t="n">
+      <c r="A34" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B34" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D34" s="6" t="s">
-        <v>91</v>
+        <v>117</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>92</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B35" s="9" t="n">
+      <c r="A35" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B35" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D35" s="6" t="s">
-        <v>92</v>
+        <v>117</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B36" s="9" t="n">
+      <c r="A36" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B36" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D36" s="6" t="s">
-        <v>93</v>
+        <v>117</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B37" s="9" t="n">
+      <c r="A37" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B37" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D37" s="6" t="s">
-        <v>94</v>
+        <v>117</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B38" s="9" t="n">
+      <c r="A38" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B38" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D38" s="6" t="s">
-        <v>95</v>
+        <v>117</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>96</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="8" t="n">
-        <v>45372</v>
-      </c>
-      <c r="B39" s="9" t="n">
+      <c r="A39" s="7" t="n">
+        <v>45372</v>
+      </c>
+      <c r="B39" s="8" t="n">
         <v>45377</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="D39" s="6" t="s">
-        <v>96</v>
+        <v>117</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>